<commit_message>
deploy: feature/careteam → branches/feature-careteam 7d08014bf24f3dbc7535181b4311c76900c8a147
</commit_message>
<xml_diff>
--- a/branches/feature-careteam/CodeSystem-typ-av-fast-kontakt-cs.xlsx
+++ b/branches/feature-careteam/CodeSystem-typ-av-fast-kontakt-cs.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="57">
   <si>
     <t>Property</t>
   </si>
@@ -66,7 +66,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-15T09:21:11+00:00</t>
+    <t>2026-10-15T12:03:42+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -126,52 +126,64 @@
     <t>Count</t>
   </si>
   <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Display</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>fast vårdkontakt</t>
+  </si>
+  <si>
+    <t>namngiven personal inom hälso- och sjukvård som ska bistå och stödja patienten genom att samordna vårdens insatser och övriga kontakter</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>fast läkarkontakt i primärvård</t>
+  </si>
+  <si>
+    <t>namngiven läkare på den hälso- eller vårdcentral där patienten är listad, som ansvarar för och samordnar patientens medicinska vård</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>fast omsorgskontakt i hemtjänsten</t>
+  </si>
+  <si>
+    <t>namngiven personal inom hemtjänstens verkställande verksamhet som ska bistå och stödja omsorgstagaren och hens anhöriga genom att samordna insatser och övriga kontakter</t>
+  </si>
+  <si>
     <t>4</t>
   </si>
   <si>
-    <t>Level</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>Display</t>
-  </si>
-  <si>
-    <t>Definition</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>fast vårdkontakt</t>
-  </si>
-  <si>
-    <t>namngiven personal inom hälso- och sjukvård som ska bistå och stödja patienten genom att samordna vårdens insatser och övriga kontakter</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>fast läkarkontakt i primärvård</t>
-  </si>
-  <si>
-    <t>namngiven läkare på den hälso- eller vårdcentral där patienten är listad, som ansvarar för och samordnar patientens medicinska vård</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>fast omsorgskontakt i hemtjänsten</t>
-  </si>
-  <si>
-    <t>namngiven personal inom hemtjänstens verkställande verksamhet som ska bistå och stödja omsorgstagaren och hens anhöriga genom att samordna insatser och övriga kontakter</t>
-  </si>
-  <si>
     <t>fast vårdkontakt med övergripande samordningsansvar</t>
   </si>
   <si>
     <t>en fast vårdkontakt med övergripande ansvar för samordning, i de fall en patient har flera fasta vårdkontakter</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>annan fast kontakt</t>
+  </si>
+  <si>
+    <t>namngiven personal inom hälso- och sjukvård eller omsorg som ska bistå och stödja patienten eller omsorgstagaren genom att samordna insatser och kontakter, men som inte motsvarar någon av de särskilt angivna typerna av fast kontakt</t>
   </si>
 </sst>
 </file>
@@ -487,7 +499,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -551,13 +563,27 @@
         <v>42</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s" s="2">
+        <v>54</v>
+      </c>
+      <c r="C6" t="s" s="2">
+        <v>55</v>
+      </c>
+      <c r="D6" t="s" s="2">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>